<commit_message>
Add Github Actions workflow files
</commit_message>
<xml_diff>
--- a/test-data/testData.xlsx
+++ b/test-data/testData.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tejavathidoddapaneni/MaextroAutomationTests/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36BA0FBE-D50D-9F42-B77A-CBD595A293B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94CD9BEF-EB8D-B54D-9282-7FDED23CFE26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{1DB15CAB-000F-BE45-BA54-865C07A11F06}"/>
   </bookViews>
   <sheets>
     <sheet name="Request" sheetId="2" r:id="rId1"/>
-    <sheet name="BOR1" sheetId="1" r:id="rId2"/>
-    <sheet name="BP00" sheetId="3" r:id="rId3"/>
-    <sheet name="KOR1" sheetId="4" r:id="rId4"/>
-    <sheet name="KOR2" sheetId="5" r:id="rId5"/>
-    <sheet name="BP01" sheetId="6" r:id="rId6"/>
-    <sheet name="BP10" sheetId="7" r:id="rId7"/>
-    <sheet name="BP11" sheetId="8" r:id="rId8"/>
-    <sheet name="BP12" sheetId="9" r:id="rId9"/>
-    <sheet name="BP07" sheetId="10" r:id="rId10"/>
+    <sheet name="Sheet1" sheetId="11" r:id="rId2"/>
+    <sheet name="BOR1" sheetId="1" r:id="rId3"/>
+    <sheet name="BP00" sheetId="3" r:id="rId4"/>
+    <sheet name="KOR1" sheetId="4" r:id="rId5"/>
+    <sheet name="KOR2" sheetId="5" r:id="rId6"/>
+    <sheet name="BP01" sheetId="6" r:id="rId7"/>
+    <sheet name="BP10" sheetId="7" r:id="rId8"/>
+    <sheet name="BP11" sheetId="8" r:id="rId9"/>
+    <sheet name="BP12" sheetId="9" r:id="rId10"/>
+    <sheet name="BP07" sheetId="10" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="664" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="166">
   <si>
     <t>Mandatory</t>
   </si>
@@ -479,36 +480,9 @@
     <t>X0001</t>
   </si>
   <si>
-    <t>STEP NO</t>
-  </si>
-  <si>
-    <t>TASK TYPE</t>
-  </si>
-  <si>
-    <t>VIEWS</t>
-  </si>
-  <si>
-    <t>CREATE_REQUEST</t>
-  </si>
-  <si>
-    <t>BD1, BD2, ORG1, ORG2</t>
-  </si>
-  <si>
-    <t>DATA</t>
-  </si>
-  <si>
-    <t>BD1, MRP</t>
-  </si>
-  <si>
-    <t>BD1, PUR</t>
-  </si>
-  <si>
     <t>DATA APPROVAL</t>
   </si>
   <si>
-    <t>BD1, ORG1, ORG2, MRP, PUR</t>
-  </si>
-  <si>
     <t>view</t>
   </si>
   <si>
@@ -555,6 +529,21 @@
   </si>
   <si>
     <t>Data Collection</t>
+  </si>
+  <si>
+    <t>BOR1,BP00,KOR1,KOR2</t>
+  </si>
+  <si>
+    <t>BP10,BP11</t>
+  </si>
+  <si>
+    <t>BOR1,BP01</t>
+  </si>
+  <si>
+    <t>BP07</t>
+  </si>
+  <si>
+    <t>Workflow Action</t>
   </si>
 </sst>
 </file>
@@ -973,14 +962,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3D1E805-262A-FB4E-9901-9967BEF52482}">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="47.1640625" customWidth="1"/>
-    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36" customWidth="1"/>
     <col min="6" max="7" width="23.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1166,164 +1155,45 @@
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>143</v>
-      </c>
-      <c r="B18" t="s">
-        <v>164</v>
-      </c>
-      <c r="C18" t="s">
-        <v>16</v>
-      </c>
-      <c r="D18" t="s">
-        <v>18</v>
-      </c>
-      <c r="E18" t="s">
-        <v>19</v>
-      </c>
-      <c r="F18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" s="7" t="s">
-        <v>165</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A22" s="7" t="s">
-        <v>166</v>
-      </c>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="7"/>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="7"/>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="7"/>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A27" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>145</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A28" s="7">
-        <v>0</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="7">
-        <v>100</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A30" s="7">
-        <v>200</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>149</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A31" s="7">
-        <v>300</v>
-      </c>
-      <c r="B31" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>153</v>
-      </c>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" s="7"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" s="7"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" s="7"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" s="7"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" s="7"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1331,6 +1201,231 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F69736E5-70CA-D145-9D1F-2E2D4B50031B}">
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s">
+        <v>4</v>
+      </c>
+      <c r="H2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" t="s">
+        <v>4</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G3" t="s">
+        <v>5</v>
+      </c>
+      <c r="H3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="F7" t="s">
+        <v>130</v>
+      </c>
+      <c r="G7" t="s">
+        <v>131</v>
+      </c>
+      <c r="H7" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <v>2</v>
+      </c>
+      <c r="F8" t="s">
+        <v>130</v>
+      </c>
+      <c r="G8" t="s">
+        <v>133</v>
+      </c>
+      <c r="H8" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>1</v>
+      </c>
+      <c r="B11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <v>2</v>
+      </c>
+      <c r="B12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" t="s">
+        <v>47</v>
+      </c>
+      <c r="E12" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F78CA850-DE65-B64D-A5D8-3376848DFFD1}">
   <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1681,8 +1776,185 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{887451B3-A29C-6D4B-8FD6-3F7EA12D0F42}">
+  <dimension ref="A7:G23"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>143</v>
+      </c>
+      <c r="B8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="187" x14ac:dyDescent="0.2">
+      <c r="A13" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="C13" t="s">
+        <v>137</v>
+      </c>
+      <c r="D13" t="s">
+        <v>137</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A6A686D-AE76-D741-9DC1-986AFAFBC071}">
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="13.1640625" bestFit="1" customWidth="1"/>
@@ -1811,69 +2083,13 @@
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>158</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="7" t="s">
-        <v>160</v>
-      </c>
-      <c r="B21" s="7" t="s">
-        <v>161</v>
-      </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4073B51-196A-7043-A35A-5E5758356E46}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2038,7 +2254,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9D8E8C6-D65B-4443-AE4E-658402AAAD1E}">
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2197,7 +2413,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35A89E81-FFF2-6841-84ED-3204DC10E603}">
   <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2399,7 +2615,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2E4BB7F-B06B-8045-B0E8-C08CBFCDC914}">
   <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -2868,7 +3084,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4842F62D-59E5-9544-B888-AD05DBFF50B0}">
   <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3191,7 +3407,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{947F56A1-7388-534A-977C-0D5C52A0D8F0}">
   <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3389,229 +3605,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F69736E5-70CA-D145-9D1F-2E2D4B50031B}">
-  <dimension ref="A1:H12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="18.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.83203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.5" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" t="s">
-        <v>5</v>
-      </c>
-      <c r="F2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" t="s">
-        <v>4</v>
-      </c>
-      <c r="H2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" t="s">
-        <v>4</v>
-      </c>
-      <c r="E3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" t="s">
-        <v>6</v>
-      </c>
-      <c r="G4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>1</v>
-      </c>
-      <c r="F7" t="s">
-        <v>130</v>
-      </c>
-      <c r="G7" t="s">
-        <v>131</v>
-      </c>
-      <c r="H7" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>2</v>
-      </c>
-      <c r="F8" t="s">
-        <v>130</v>
-      </c>
-      <c r="G8" t="s">
-        <v>133</v>
-      </c>
-      <c r="H8" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>1</v>
-      </c>
-      <c r="B11" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>2</v>
-      </c>
-      <c r="B12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" t="s">
-        <v>48</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>